<commit_message>
feat: se han mejorado algunas traducciones
</commit_message>
<xml_diff>
--- a/lib/l10n/translation_log.xlsx
+++ b/lib/l10n/translation_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -499,6 +499,1388 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:09:46</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Logged in successfully</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>auth_login_success</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:12:19</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Cloud Backup</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>settings_cloud_backup</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:12:42</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Migrate from Joss Music Kotlin</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>settings_migration_title</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:13:01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Do you want to perform a backup?</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>backup_confirm_question</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:13:23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Choose which data to backup</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>backup_selection_prompt</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:14:39</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Búsquedas recientes</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>search_recent_title</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:17:25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sesión iniciada correctamente</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>auth_login_success</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:17:38</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Volver</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:18:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Olvidé mi contraseña</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>auth_forgot_password</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:18:17</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Iniciar sesión</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>auth_btn_login</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:18:30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Registrarme</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>auth_btn_register</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:18:45</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:19:09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Password</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>password_text</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Contraseña texto traducido</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:19:27</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Confirmar contraseña</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>auth_confirm_password</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:19:51</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Welcome to Estrella Music</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>auth_welcome_title</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:20:09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Accede con tu cuenta...</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Welcome to Estrella Music</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>auth_welcome_subtitle</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:20:52</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Username</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>username</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:22:11</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>First name</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>auth_first_name</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:22:25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Last name</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>auth_last_name</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:22:41</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Acepto usar mis datos...</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>auth_agree_personal_data</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:22:56</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>settings_general_section</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:23:14</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Cerrar sesion</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>settings_logout</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:23:32</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Backup en la nube</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>settings_cloud_backup</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:24:17</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Sube, restaura y administra...</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>settings_cloud_backup_desc</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:24:33</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Migrar desde Joss Music Kotlin</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>settings_migration_title</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:24:50</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Importa playlists, canciones...</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>settings_migration_desc</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:25:23</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Reiniciar app</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>backup_btn_restart</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:25:40</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Subir backup ahora</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>backup_btn_upload</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:26:02</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Todavía no hay backups...</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>backup_no_backups</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:26:18</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Necesitas una sesión activa...</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>backup_auth_required</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:26:37</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Backup subido correctamente.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>backup_upload_success</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:26:54</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Backup restaurado. Reinicia la app.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>backup_restore_success</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:27:10</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Backup eliminado.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>backup_delete_success</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:27:33</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Búsquedas recientes</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>search_recent_title</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:27:50</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Pop</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>genre_pop</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:28:04</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Rock</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>genre_rock</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:28:28</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Hip Hop</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>genre_hiphop</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:28:47</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Electronic</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>genre_electronic</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:29:18</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Electrónica</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>genre_electronic</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:29:45</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Jazz</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>genre_jazz</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:30:01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Latin</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>genre_latin</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:30:19</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Seleccionar archivo e importar</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>migration_btn_select</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-03-30 20:30:35</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Cerrar</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>close</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Nuevo diseño M3E directo
</commit_message>
<xml_diff>
--- a/lib/l10n/translation_log.xlsx
+++ b/lib/l10n/translation_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1869,13 +1869,333 @@
           <t>close</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>Traducción y Adición</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:37:17</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Favoritos olvidados</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>forgottenFavorites</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:41:02</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>La canción más escuchada</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>mostListenedSong</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:41:43</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Reproducida por</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>reproducedBy</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:42:23</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Búsquedas recientes</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>recentSearches</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-05-07 22:45:24</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Pistas populares</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>popularTracks</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-05-07 22:47:14</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Último lanzamiento</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>latestRelease</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-05-07 22:47:34</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Seguir</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>follow</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-05-07 22:47:52</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Siguiendo</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>following</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-05-07 22:48:05</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Escuchar ahora</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>listenNow</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-05-07 22:48:22</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
         <is>
           <t>flutter</t>
         </is>

</xml_diff>

<commit_message>
feat: Mejoras en traducciones y quitamos residuos de Harmony Music
</commit_message>
<xml_diff>
--- a/lib/l10n/translation_log.xlsx
+++ b/lib/l10n/translation_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2189,13 +2189,109 @@
           <t>video</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>Traducción y Adición</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-05-10 23:07:02</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Acerca de</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>about</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-05-10 23:08:26</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Acerca de</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>about</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-05-10 23:11:23</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Leer más</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>readMore</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
         <is>
           <t>flutter</t>
         </is>

</xml_diff>

<commit_message>
feat: Mejoras en el diseño del reproductor, traducciones y listas
</commit_message>
<xml_diff>
--- a/lib/l10n/translation_log.xlsx
+++ b/lib/l10n/translation_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2285,13 +2285,525 @@
           <t>readMore</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>Traducción y Adición</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:14:39</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Velocidad y Tono</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>speedAndPitch</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:14:55</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Velocidad de reproducción</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>playbackSpeed</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:15:23</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Tono de la canción</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>songPitch</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:15:40</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Reconocimiento de Música</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>musicRecognition</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:15:56</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Escuchando el entorno...</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>listeningToEnvironment</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:16:13</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Asegúrate de que la música suene con suficiente volumen cerca de tu micrófono.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>micInstruction</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:16:30</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Procesando el audio...</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>processingAudio</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:16:48</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Buscando coincidencias en la base de datos de Shazam...</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>shazamSearching</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:17:04</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>¡Canción Encontrada!</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>songFound</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:17:20</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Reproducir Ahora</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>playNow</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:17:36</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Buscar en Biblioteca</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>searchInLibrary</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:17:51</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Sin Coincidencias</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>noMatchesFound</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:18:08</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>No se pudo encontrar ninguna canción en el audio registrado</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>noMatchInstruction</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:18:27</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Ocurrió un error</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>errorOccurred</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:18:44</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Reproduciendo:</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>playingRecognizedTrack</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-05-17 20:18:59</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Error al reproducir:</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>errorPlayingTrack</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Traducción y Adición</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
         <is>
           <t>flutter</t>
         </is>

</xml_diff>